<commit_message>
scan: seg8 2026-08-07 17:02 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-08-07.xlsx
+++ b/output/full_scan/batch_seq0_2026-08-07.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O116"/>
+  <dimension ref="A1:O117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5986,38 +5986,38 @@
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>8201</v>
+        <v>8291</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>無敵</t>
+          <t>尚茂</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>153.0833145496609</v>
+        <v>157.6356845468096</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>11.85</v>
+        <v>41</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="G105" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>41.45194262660245</v>
+        <v>51.64457685049216</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>27.29063900058471</v>
+        <v>16.15980708385423</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.5003096098915366</v>
+        <v>0.7772094107632718</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0095391533111018</v>
+        <v>0.9275611706969576</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8072</v>
+        <v>8201</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>陞泰</t>
+          <t>無敵</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>152.4279261332631</v>
+        <v>153.0833145496609</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>26.2</v>
+        <v>11.85</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>40.02614605174998</v>
+        <v>41.45194262660245</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>18.85194147237907</v>
+        <v>27.29063900058471</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1.201002637853382</v>
+        <v>0.5003096098915366</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.003120956685825</v>
+        <v>-0.0095391533111018</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>9902</v>
+        <v>8072</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>台火</t>
+          <t>陞泰</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>151.5889144445398</v>
+        <v>152.4279261332631</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>13.65</v>
+        <v>26.2</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>48.28544192160889</v>
+        <v>40.02614605174998</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>8.380322325980716</v>
+        <v>18.85194147237907</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>1.004579451418339</v>
+        <v>1.201002637853382</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.0041992038716511</v>
+        <v>0.003120956685825</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6145,38 +6145,38 @@
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>8455</v>
+        <v>9902</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>大拓-KY</t>
+          <t>台火</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>151.0844712337206</v>
+        <v>151.5889144445398</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>24</v>
+        <v>13.65</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G108" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>41.23986164140064</v>
+        <v>48.28544192160889</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>18.02251253302201</v>
+        <v>8.380322325980716</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.2037479434191961</v>
+        <v>1.004579451418339</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,48 +6188,48 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.0644627860794218</v>
+        <v>0.0041992038716511</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>8341</v>
+        <v>8455</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>日友</t>
+          <t>大拓-KY</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>147.7904802489458</v>
+        <v>151.0844712337206</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>75.3</v>
+        <v>24</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="G109" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>42.56493332330227</v>
+        <v>41.23986164140064</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>13.4632965375826</v>
+        <v>18.02251253302201</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.3995782710820679</v>
+        <v>0.2037479434191961</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,48 +6241,48 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.07622855567564379</v>
+        <v>0.0644627860794218</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8091</v>
+        <v>8341</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>翔名</t>
+          <t>日友</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>146.6491692746877</v>
+        <v>147.7904802489458</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>225</v>
+        <v>75.3</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G110" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>43.85707942618112</v>
+        <v>42.56493332330227</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>18.0500211690647</v>
+        <v>13.4632965375826</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.2989810132885925</v>
+        <v>0.3995782710820679</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,51 +6294,51 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.7618913093330217</v>
+        <v>-0.07622855567564379</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>8940</v>
+        <v>8091</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>新天地</t>
+          <t>翔名</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>139.753827533148</v>
+        <v>146.6491692746877</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>15.35</v>
+        <v>225</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="G111" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>26.0091718586589</v>
+        <v>43.85707942618112</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>16.71545151585148</v>
+        <v>18.0500211690647</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.4870141824879453</v>
+        <v>0.2989810132885925</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.0535666183175262</v>
+        <v>-0.7618913093330217</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>8104</v>
+        <v>8940</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>錸寶</t>
+          <t>新天地</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>101.6916263052699</v>
+        <v>139.753827533148</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>31.15</v>
+        <v>15.35</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>38.6551616894116</v>
+        <v>26.0091718586589</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>31.29975891663564</v>
+        <v>16.71545151585148</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.3373780161006777</v>
+        <v>0.4870141824879453</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,48 +6400,48 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1040917482604428</v>
+        <v>-0.0535666183175262</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>8176</v>
+        <v>8104</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>智捷</t>
+          <t>錸寶</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>99.81943247202231</v>
+        <v>101.6916263052699</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>9.779999999999999</v>
+        <v>31.15</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="G113" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>42.26924979224129</v>
+        <v>38.6551616894116</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>9.790890624006884</v>
+        <v>31.29975891663564</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.5699220552814119</v>
+        <v>0.3373780161006777</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.0042802299970707</v>
+        <v>-0.1040917482604428</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>8068</v>
+        <v>8176</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>全達</t>
+          <t>智捷</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>98.99222743633622</v>
+        <v>99.81943247202231</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>17.9</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>46.63522593072307</v>
+        <v>42.26924979224129</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>16.60510234072982</v>
+        <v>9.790890624006884</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.4060210808821017</v>
+        <v>0.5699220552814119</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0664319527525452</v>
+        <v>-0.0042802299970707</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6516,21 +6516,21 @@
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>8076</v>
+        <v>8068</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>伍豐</t>
+          <t>全達</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>88.02841556185359</v>
+        <v>98.99222743633622</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>23.15</v>
+        <v>17.9</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>44.6272877605498</v>
+        <v>46.63522593072307</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>13.33895280961058</v>
+        <v>16.60510234072982</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.4038049544714736</v>
+        <v>0.4060210808821017</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.0605746476931836</v>
+        <v>0.0664319527525452</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6569,52 +6569,105 @@
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
+        <v>8076</v>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>伍豐</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D116" s="2" t="n">
+        <v>88.02841556185359</v>
+      </c>
+      <c r="E116" s="2" t="n">
+        <v>23.15</v>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H116" s="2" t="n">
+        <v>44.6272877605498</v>
+      </c>
+      <c r="I116" s="2" t="n">
+        <v>13.33895280961058</v>
+      </c>
+      <c r="J116" s="2" t="n">
+        <v>0.4038049544714736</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M116" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N116" s="2" t="n">
+        <v>0.0605746476931836</v>
+      </c>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="n">
         <v>9906</v>
       </c>
-      <c r="B116" s="2" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>欣巴巴</t>
         </is>
       </c>
-      <c r="C116" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D116" s="2" t="n">
+      <c r="C117" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D117" s="2" t="n">
         <v>61.70488338832593</v>
       </c>
-      <c r="E116" s="2" t="n">
+      <c r="E117" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="F116" s="2" t="inlineStr">
+      <c r="F117" s="2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="G116" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H116" s="2" t="n">
+      <c r="G117" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H117" s="2" t="n">
         <v>44.00728499973047</v>
       </c>
-      <c r="I116" s="2" t="n">
+      <c r="I117" s="2" t="n">
         <v>11.51247174193982</v>
       </c>
-      <c r="J116" s="2" t="n">
+      <c r="J117" s="2" t="n">
         <v>0.5054175002599628</v>
       </c>
-      <c r="K116" s="2" t="n">
+      <c r="K117" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L116" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M116" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N116" s="2" t="n">
+      <c r="L117" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M117" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N117" s="2" t="n">
         <v>-0.1084879191291834</v>
       </c>
-      <c r="O116" s="2" t="inlineStr">
+      <c r="O117" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>